<commit_message>
Update Variable List 2021 Data sheet from Senegal to Benin
- Replace all _sen2021 dataset names with _ben2021
- Update title from EHCVM Senegal 2021 to EHCVM Benin 2021
- s10q61a: extend HH member range from 8 to 9 (Benin has up to 9)
- s04q38: update formality indicator label from IPRES/FNR to FNRB/CNSS
- Remove zali0 (food poverty line not present in Benin 2021 welfare)
- Move shock variables (sh_id_demo–sh_co_oth) from welfare section to
  menage section (they come from ehcvm_menage_ben2021, not welfare)
- Remove region from menage section (not in Benin 2021 menage file)
- Move milieu from menage section to welfare section
- Add departement to welfare section (Benin uses departement not region)
- Update section descriptions to reflect Benin 2021 data structure

https://claude.ai/code/session_01CRdVYRGorJ7cRR6RNWekdA
</commit_message>
<xml_diff>
--- a/Output/Variable List.xlsx
+++ b/Output/Variable List.xlsx
@@ -4165,8 +4165,8 @@
     <mergeCell ref="A75:D75"/>
     <mergeCell ref="A101:D101"/>
     <mergeCell ref="A210:D210"/>
+    <mergeCell ref="A95:D95"/>
     <mergeCell ref="A76:D76"/>
-    <mergeCell ref="A95:D95"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
@@ -4186,7 +4186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D243"/>
+  <dimension ref="A1:D242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" style="5" min="1" max="1"/>
@@ -4197,7 +4197,7 @@
     <row r="1" ht="18.75" customHeight="1" s="5">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>EHCVM Senegal 2021 — Raw Variables Used in 03_clean_2021.do</t>
+          <t>EHCVM Benin 2021 — Raw Variables Used in 03_clean_2021.do</t>
         </is>
       </c>
     </row>
@@ -4208,6 +4208,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15.75" customHeight="1" s="5">
       <c r="A4" s="1" t="inlineStr">
         <is>
@@ -4233,7 +4234,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Section 10B — Enterprise Details  |  Dataset: s10b_me_sen2021</t>
+          <t>Section 10B — Enterprise Details  |  Dataset: s10b_me_ben2021</t>
         </is>
       </c>
     </row>
@@ -4356,12 +4357,12 @@
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>s10q61a_1 to s10q61a_8</t>
+          <t>s10q61a_1 to s10q61a_9</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Code ID of HH member working in enterprise (up to 8; was 14 in 2018)</t>
+          <t>Code ID of HH member working in enterprise (up to 9; was 14 in 2018)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -5270,10 +5271,11 @@
         </is>
       </c>
     </row>
+    <row r="64"/>
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>Section 10A — Enterprise Screening  |  Dataset: s10a_me_sen2021</t>
+          <t>Section 10A — Enterprise Screening  |  Dataset: s10a_me_ben2021</t>
         </is>
       </c>
     </row>
@@ -5446,10 +5448,11 @@
         </is>
       </c>
     </row>
+    <row r="76"/>
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>ehcvm_individu — Individual Characteristics  |  Dataset: ehcvm_individu_sen2021</t>
+          <t>ehcvm_individu — Individual Characteristics  |  Dataset: ehcvm_individu_ben2021</t>
         </is>
       </c>
     </row>
@@ -5784,10 +5787,11 @@
         </is>
       </c>
     </row>
+    <row r="97"/>
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>Section 4A — Employment Status (2021 split)  |  Dataset: s04a_me_sen2021</t>
+          <t>Section 4A — Employment Status (2021 split)  |  Dataset: s04a_me_ben2021</t>
         </is>
       </c>
     </row>
@@ -6014,10 +6018,11 @@
         </is>
       </c>
     </row>
+    <row r="112"/>
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>Section 4B — Primary Job Details (2021 split)  |  Dataset: s04b_me_sen2021</t>
+          <t>Section 4B — Primary Job Details (2021 split)  |  Dataset: s04b_me_ben2021</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6150,7 @@
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>Contributes to IPRES/FNR/Retraite (formality indicator — NEW in 2021 cleaning)</t>
+          <t>Contributes to FNRB/CNSS (formality indicator — NEW in 2021 cleaning)</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -6406,10 +6411,11 @@
         </is>
       </c>
     </row>
+    <row r="136"/>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>Section 4C — Secondary Job Details (2021 split)  |  Dataset: s04c_me_sen2021</t>
+          <t>Section 4C — Secondary Job Details (2021 split)  |  Dataset: s04c_me_ben2021</t>
         </is>
       </c>
     </row>
@@ -6708,17 +6714,18 @@
         </is>
       </c>
     </row>
+    <row r="155"/>
     <row r="156">
       <c r="A156" s="6" t="inlineStr">
         <is>
-          <t>ehcvm_menage — Household Characteristics  |  Dataset: ehcvm_menage_sen2021</t>
+          <t>ehcvm_menage — Household Characteristics  |  Dataset: ehcvm_menage_ben2021</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
         <is>
-          <t>Housing conditions, assets, and household demographics (same structure as 2018)</t>
+          <t>Housing conditions, assets, and household demographics. In Benin 2021, shock variables (sh_id_demo–sh_co_oth) are sourced from this file (not from welfare).</t>
         </is>
       </c>
     </row>
@@ -7194,17 +7201,17 @@
       <c r="A184" s="2" t="n"/>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>sh_id_demo</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Administrative region</t>
+          <t>Idiosyncratic demographic shock (illness, death)</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>Region residence</t>
+          <t>Choc idio démographique</t>
         </is>
       </c>
     </row>
@@ -7212,31 +7219,71 @@
       <c r="A185" s="2" t="n"/>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>milieu</t>
+          <t>sh_co_natu</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>Urban/Rural</t>
+          <t>Covariate natural shock (flood, drought)</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>Milieu residence</t>
+          <t>Choc covariant naturel</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="n"/>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>sh_co_eco</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Covariate economic shock (price increase)</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>Choc covariant économique</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="6" t="inlineStr">
-        <is>
-          <t>ehcvm_welfare — Welfare and Consumption Aggregates  |  Dataset: ehcvm_welfare_sen2021</t>
+      <c r="A187" s="2" t="n"/>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>sh_id_eco</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Idiosyncratic economic shock (job loss)</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>Choc idio économique</t>
         </is>
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="4" t="inlineStr">
-        <is>
-          <t>Pre-constructed welfare measures. 2021 has additional deflator variables.</t>
+      <c r="A188" s="2" t="n"/>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>sh_co_vio</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>Violence/conflict shock</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Choc covariant violence</t>
         </is>
       </c>
     </row>
@@ -7244,71 +7291,32 @@
       <c r="A189" s="2" t="n"/>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>hhsize</t>
+          <t>sh_co_oth</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>Household size</t>
+          <t>Other shock</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>Taille menage</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="2" t="n"/>
-      <c r="B190" s="2" t="inlineStr">
-        <is>
-          <t>eqadu1</t>
-        </is>
-      </c>
-      <c r="C190" s="2" t="inlineStr">
-        <is>
-          <t>Adult equivalent scale 1</t>
-        </is>
-      </c>
-      <c r="D190" s="2" t="inlineStr">
-        <is>
-          <t>Nbr adultes-equiv. FAO</t>
-        </is>
-      </c>
-    </row>
+          <t>Autres Chocs</t>
+        </is>
+      </c>
+    </row>
+    <row r="190"/>
     <row r="191">
-      <c r="A191" s="2" t="n"/>
-      <c r="B191" s="2" t="inlineStr">
-        <is>
-          <t>eqadu2</t>
-        </is>
-      </c>
-      <c r="C191" s="2" t="inlineStr">
-        <is>
-          <t>Adult equivalent scale 2</t>
-        </is>
-      </c>
-      <c r="D191" s="2" t="inlineStr">
-        <is>
-          <t>Nbr adultes-equiv. alt.</t>
+      <c r="A191" s="6" t="inlineStr">
+        <is>
+          <t>ehcvm_welfare — Welfare and Consumption Aggregates  |  Dataset: ehcvm_welfare_ben2021</t>
         </is>
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n"/>
-      <c r="B192" s="2" t="inlineStr">
-        <is>
-          <t>dali</t>
-        </is>
-      </c>
-      <c r="C192" s="2" t="inlineStr">
-        <is>
-          <t>Food consumption aggregate</t>
-        </is>
-      </c>
-      <c r="D192" s="2" t="inlineStr">
-        <is>
-          <t>Conso annuelle alim. menage</t>
+      <c r="A192" s="4" t="inlineStr">
+        <is>
+          <t>Pre-constructed welfare measures. 2021 has additional deflator variables. In Benin 2021, geographic vars (departement, milieu) come from this file (shocks are in menage).</t>
         </is>
       </c>
     </row>
@@ -7316,17 +7324,17 @@
       <c r="A193" s="2" t="n"/>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>dnal</t>
+          <t>hhsize</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Non-food consumption aggregate</t>
+          <t>Household size</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>Conso annuelle non alim. menage</t>
+          <t>Taille menage</t>
         </is>
       </c>
     </row>
@@ -7334,17 +7342,17 @@
       <c r="A194" s="2" t="n"/>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>dtot</t>
+          <t>eqadu1</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Total consumption aggregate</t>
+          <t>Adult equivalent scale 1</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>Conso annuelle totale menage</t>
+          <t>Nbr adultes-equiv. FAO</t>
         </is>
       </c>
     </row>
@@ -7352,17 +7360,17 @@
       <c r="A195" s="2" t="n"/>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>pcexp</t>
+          <t>eqadu2</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Per capita expenditure</t>
+          <t>Adult equivalent scale 2</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>Indicateur de bien-être</t>
+          <t>Nbr adultes-equiv. alt.</t>
         </is>
       </c>
     </row>
@@ -7370,31 +7378,35 @@
       <c r="A196" s="2" t="n"/>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>zzae</t>
+          <t>dali</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Agro-ecological zone (welfare file)</t>
-        </is>
-      </c>
-      <c r="D196" s="2" t="n"/>
+          <t>Food consumption aggregate</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Conso annuelle alim. menage</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n"/>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>zref</t>
+          <t>dnal</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Poverty line</t>
+          <t>Non-food consumption aggregate</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>Seuil pauvrete national</t>
+          <t>Conso annuelle non alim. menage</t>
         </is>
       </c>
     </row>
@@ -7402,17 +7414,17 @@
       <c r="A198" s="2" t="n"/>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>def_spa</t>
+          <t>dtot</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Spatial price deflator</t>
+          <t>Total consumption aggregate</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>Deflateur spatial</t>
+          <t>Conso annuelle totale menage</t>
         </is>
       </c>
     </row>
@@ -7420,17 +7432,17 @@
       <c r="A199" s="2" t="n"/>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>def_temp</t>
+          <t>pcexp</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Temporal price deflator</t>
+          <t>Per capita expenditure</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>Deflateur temporel</t>
+          <t>Indicateur de bien-être</t>
         </is>
       </c>
     </row>
@@ -7438,35 +7450,31 @@
       <c r="A200" s="2" t="n"/>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>def_temp_prix2021m11</t>
-        </is>
-      </c>
-      <c r="C200" s="3" t="inlineStr">
-        <is>
-          <t>Temporal deflator based on Nov 2021 prices (NEW in 2021)</t>
-        </is>
-      </c>
-      <c r="D200" s="2" t="inlineStr">
-        <is>
-          <t>temporal deflator for international poverty, 1 = 2021m11 prices</t>
-        </is>
-      </c>
+          <t>zzae</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Agro-ecological zone (welfare file)</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n"/>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>def_temp_cpi</t>
-        </is>
-      </c>
-      <c r="C201" s="3" t="inlineStr">
-        <is>
-          <t>CPI-based temporal deflator (NEW in 2021)</t>
+          <t>departement</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>Administrative department</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>alternative temporal deflator based on official CPI, 2018/19 style</t>
+          <t>Departement residence</t>
         </is>
       </c>
     </row>
@@ -7474,17 +7482,17 @@
       <c r="A202" s="2" t="n"/>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>def_temp_adj</t>
-        </is>
-      </c>
-      <c r="C202" s="3" t="inlineStr">
-        <is>
-          <t>Adjusted temporal deflator (NEW in 2021)</t>
+          <t>milieu</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Urban/Rural</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>temporal deflator adjusted for difference between hh and market survey periods</t>
+          <t>Milieu residence</t>
         </is>
       </c>
     </row>
@@ -7492,17 +7500,17 @@
       <c r="A203" s="2" t="n"/>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>zali0</t>
-        </is>
-      </c>
-      <c r="C203" s="3" t="inlineStr">
-        <is>
-          <t>Food poverty line (NEW in 2021)</t>
+          <t>zref</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>Poverty line</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>(sum) conso_pc_val_up</t>
+          <t>Seuil pauvrete national</t>
         </is>
       </c>
     </row>
@@ -7510,31 +7518,35 @@
       <c r="A204" s="2" t="n"/>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>dtet</t>
-        </is>
-      </c>
-      <c r="C204" s="3" t="inlineStr">
-        <is>
-          <t>Total consumption (alternative) (NEW in 2021)</t>
-        </is>
-      </c>
-      <c r="D204" s="2" t="n"/>
+          <t>def_spa</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>Spatial price deflator</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Deflateur spatial</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n"/>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>monthly_cpi</t>
-        </is>
-      </c>
-      <c r="C205" s="3" t="inlineStr">
-        <is>
-          <t>Monthly CPI (NEW in 2021)</t>
+          <t>def_temp</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>Temporal price deflator</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>Monthly CPI value</t>
+          <t>Deflateur temporel</t>
         </is>
       </c>
     </row>
@@ -7542,45 +7554,53 @@
       <c r="A206" s="2" t="n"/>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>cpi2017</t>
+          <t>def_temp_prix2021m11</t>
         </is>
       </c>
       <c r="C206" s="3" t="inlineStr">
         <is>
-          <t>CPI base 2017 (NEW in 2021)</t>
-        </is>
-      </c>
-      <c r="D206" s="2" t="n"/>
+          <t>Temporal deflator based on Nov 2021 prices (NEW in 2021)</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>temporal deflator for international poverty, 1 = 2021m11 prices</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n"/>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>icp2017</t>
+          <t>def_temp_cpi</t>
         </is>
       </c>
       <c r="C207" s="3" t="inlineStr">
         <is>
-          <t>ICP 2017 (NEW in 2021)</t>
-        </is>
-      </c>
-      <c r="D207" s="2" t="n"/>
+          <t>CPI-based temporal deflator (NEW in 2021)</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>alternative temporal deflator based on official CPI, 2018/19 style</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n"/>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>dollars</t>
+          <t>def_temp_adj</t>
         </is>
       </c>
       <c r="C208" s="3" t="inlineStr">
         <is>
-          <t>Dollar equivalent (NEW in 2021)</t>
+          <t>Adjusted temporal deflator (NEW in 2021)</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>welfare in 2017 PPP USD per capita per day (not spatially deflated)</t>
+          <t>temporal deflator adjusted for difference between hh and market survey periods</t>
         </is>
       </c>
     </row>
@@ -7588,35 +7608,31 @@
       <c r="A209" s="2" t="n"/>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>hgender</t>
-        </is>
-      </c>
-      <c r="C209" s="2" t="inlineStr">
-        <is>
-          <t>HH head gender</t>
-        </is>
-      </c>
-      <c r="D209" s="2" t="inlineStr">
-        <is>
-          <t>Genre du CM</t>
-        </is>
-      </c>
+          <t>dtet</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>Total consumption (alternative) (NEW in 2021)</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n"/>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>hage</t>
-        </is>
-      </c>
-      <c r="C210" s="2" t="inlineStr">
-        <is>
-          <t>HH head age</t>
+          <t>monthly_cpi</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Monthly CPI (NEW in 2021)</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>Age du CM</t>
+          <t>Monthly CPI value</t>
         </is>
       </c>
     </row>
@@ -7624,53 +7640,45 @@
       <c r="A211" s="2" t="n"/>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>hmstat</t>
-        </is>
-      </c>
-      <c r="C211" s="2" t="inlineStr">
-        <is>
-          <t>HH head marital status</t>
-        </is>
-      </c>
-      <c r="D211" s="2" t="inlineStr">
-        <is>
-          <t>Situation famille du CM</t>
-        </is>
-      </c>
+          <t>cpi2017</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>CPI base 2017 (NEW in 2021)</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n"/>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>hreligion</t>
-        </is>
-      </c>
-      <c r="C212" s="2" t="inlineStr">
-        <is>
-          <t>HH head religion</t>
-        </is>
-      </c>
-      <c r="D212" s="2" t="inlineStr">
-        <is>
-          <t>Religion du CM</t>
-        </is>
-      </c>
+          <t>icp2017</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>ICP 2017 (NEW in 2021)</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n"/>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>hnation</t>
-        </is>
-      </c>
-      <c r="C213" s="2" t="inlineStr">
-        <is>
-          <t>HH head nationality</t>
+          <t>dollars</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>Dollar equivalent (NEW in 2021)</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
         <is>
-          <t>Nationalite du CM</t>
+          <t>welfare in 2017 PPP USD per capita per day (not spatially deflated)</t>
         </is>
       </c>
     </row>
@@ -7678,17 +7686,17 @@
       <c r="A214" s="2" t="n"/>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>heduc</t>
+          <t>hgender</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>HH head education level</t>
+          <t>HH head gender</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
         <is>
-          <t>Education du CM</t>
+          <t>Genre du CM</t>
         </is>
       </c>
     </row>
@@ -7696,17 +7704,17 @@
       <c r="A215" s="2" t="n"/>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>hdiploma</t>
+          <t>hage</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>HH head diploma</t>
+          <t>HH head age</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
         <is>
-          <t>Diplome du CM</t>
+          <t>Age du CM</t>
         </is>
       </c>
     </row>
@@ -7714,17 +7722,17 @@
       <c r="A216" s="2" t="n"/>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>hhandig</t>
+          <t>hmstat</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>HH head disability</t>
+          <t>HH head marital status</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
         <is>
-          <t>Handicap majeur CM</t>
+          <t>Situation famille du CM</t>
         </is>
       </c>
     </row>
@@ -7732,17 +7740,17 @@
       <c r="A217" s="2" t="n"/>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>hactiv7j</t>
+          <t>hreligion</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>HH head activity (7 days)</t>
+          <t>HH head religion</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t>Activite 7 jours du CM</t>
+          <t>Religion du CM</t>
         </is>
       </c>
     </row>
@@ -7750,17 +7758,17 @@
       <c r="A218" s="2" t="n"/>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>hactiv12m</t>
+          <t>hnation</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>HH head activity (12 months)</t>
+          <t>HH head nationality</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t>Activite 12 mois du CM</t>
+          <t>Nationalite du CM</t>
         </is>
       </c>
     </row>
@@ -7768,17 +7776,17 @@
       <c r="A219" s="2" t="n"/>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>hbranch</t>
+          <t>heduc</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>HH head branch of activity</t>
+          <t>HH head education level</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t>Branche activite du CM</t>
+          <t>Education du CM</t>
         </is>
       </c>
     </row>
@@ -7786,17 +7794,17 @@
       <c r="A220" s="2" t="n"/>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>hsectins</t>
+          <t>hdiploma</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>HH head institutional sector</t>
+          <t>HH head diploma</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t>Secteur instit. du CM</t>
+          <t>Diplome du CM</t>
         </is>
       </c>
     </row>
@@ -7804,17 +7812,17 @@
       <c r="A221" s="2" t="n"/>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>hcsp</t>
+          <t>hhandig</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>HH head socio-professional category</t>
+          <t>HH head disability</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>CSP du CM</t>
+          <t>Handicap majeur CM</t>
         </is>
       </c>
     </row>
@@ -7822,17 +7830,17 @@
       <c r="A222" s="2" t="n"/>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>sh_id_demo</t>
+          <t>hactiv7j</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Idiosyncratic demographic shock (illness, death)</t>
+          <t>HH head activity (7 days)</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>Choc idio démographique</t>
+          <t>Activite 7 jours du CM</t>
         </is>
       </c>
     </row>
@@ -7840,17 +7848,17 @@
       <c r="A223" s="2" t="n"/>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>sh_co_natu</t>
+          <t>hactiv12m</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>Covariate natural shock (flood, drought)</t>
+          <t>HH head activity (12 months)</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>Choc covariant naturel</t>
+          <t>Activite 12 mois du CM</t>
         </is>
       </c>
     </row>
@@ -7858,17 +7866,17 @@
       <c r="A224" s="2" t="n"/>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>sh_co_eco</t>
+          <t>hbranch</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Covariate economic shock (price increase)</t>
+          <t>HH head branch of activity</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>Choc covariant économique</t>
+          <t>Branche activite du CM</t>
         </is>
       </c>
     </row>
@@ -7876,17 +7884,17 @@
       <c r="A225" s="2" t="n"/>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>sh_id_eco</t>
+          <t>hsectins</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>Idiosyncratic economic shock (job loss)</t>
+          <t>HH head institutional sector</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>Choc idio économique</t>
+          <t>Secteur instit. du CM</t>
         </is>
       </c>
     </row>
@@ -7894,49 +7902,50 @@
       <c r="A226" s="2" t="n"/>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>sh_co_vio</t>
+          <t>hcsp</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Violence/conflict shock</t>
+          <t>HH head socio-professional category</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>Choc covariant violence</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" s="2" t="n"/>
-      <c r="B227" s="2" t="inlineStr">
-        <is>
-          <t>sh_co_oth</t>
-        </is>
-      </c>
-      <c r="C227" s="2" t="inlineStr">
-        <is>
-          <t>Other shock</t>
-        </is>
-      </c>
-      <c r="D227" s="2" t="inlineStr">
-        <is>
-          <t>Autres Chocs</t>
+          <t>CSP du CM</t>
+        </is>
+      </c>
+    </row>
+    <row r="227"/>
+    <row r="228">
+      <c r="A228" s="6" t="inlineStr">
+        <is>
+          <t>Section 6 — Credit  |  Dataset: s06_me_ben2021</t>
         </is>
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="6" t="inlineStr">
-        <is>
-          <t>Section 6 — Credit  |  Dataset: s06_me_sen2021</t>
+      <c r="A229" s="4" t="inlineStr">
+        <is>
+          <t>Individual-level credit and borrowing. Note: uses 'membres__id' instead of 's01q00a' for individual ID.</t>
         </is>
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="4" t="inlineStr">
-        <is>
-          <t>Individual-level credit and borrowing. Note: uses 'membres__id' instead of 's01q00a' for individual ID.</t>
+      <c r="A230" s="2" t="n"/>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>membres__id</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>Individual ID (renamed to numind)</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>1.00. Qui est le répondant de cette section?</t>
         </is>
       </c>
     </row>
@@ -7944,17 +7953,17 @@
       <c r="A231" s="2" t="n"/>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>membres__id</t>
+          <t>s06q05</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Individual ID (renamed to numind)</t>
+          <t>Obtained credit in last 12 months?</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>1.00. Qui est le répondant de cette section?</t>
+          <t>6.05. Est-ce que [NOM] a obtenu un crédit au cours des 12 derniers mois?</t>
         </is>
       </c>
     </row>
@@ -7962,17 +7971,17 @@
       <c r="A232" s="2" t="n"/>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>s06q05</t>
+          <t>s06q12</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Obtained credit in last 12 months?</t>
+          <t>Source of credit</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>6.05. Est-ce que [NOM] a obtenu un crédit au cours des 12 derniers mois?</t>
+          <t>6.12. Auprès de qui ce dernier crédit a-t-il été contracté?</t>
         </is>
       </c>
     </row>
@@ -7980,17 +7989,17 @@
       <c r="A233" s="2" t="n"/>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>s06q12</t>
+          <t>s06q12_autre</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>Source of credit</t>
+          <t>Source of credit (other, specify)</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>6.12. Auprès de qui ce dernier crédit a-t-il été contracté?</t>
+          <t>6.12. Préciser</t>
         </is>
       </c>
     </row>
@@ -7998,17 +8007,17 @@
       <c r="A234" s="2" t="n"/>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>s06q12_autre</t>
+          <t>s06q14</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Source of credit (other, specify)</t>
+          <t>Amount of last credit (FCFA)</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>6.12. Préciser</t>
+          <t>6.14. Quel est le montant nominal de ce dernier crédit?</t>
         </is>
       </c>
     </row>
@@ -8016,17 +8025,17 @@
       <c r="A235" s="2" t="n"/>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>s06q14</t>
+          <t>s06q09</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Amount of last credit (FCFA)</t>
+          <t>Has outstanding loans from past?</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>6.14. Quel est le montant nominal de ce dernier crédit?</t>
+          <t>6.09. [NOM] a-t-il bénéficié d'1 crédit ds l passé, pas encor complet remb?</t>
         </is>
       </c>
     </row>
@@ -8034,49 +8043,50 @@
       <c r="A236" s="2" t="n"/>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>s06q09</t>
+          <t>s06q10</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Has outstanding loans from past?</t>
+          <t>Number of outstanding loans</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>6.09. [NOM] a-t-il bénéficié d'1 crédit ds l passé, pas encor complet remb?</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" s="2" t="n"/>
-      <c r="B237" s="2" t="inlineStr">
-        <is>
-          <t>s06q10</t>
-        </is>
-      </c>
-      <c r="C237" s="2" t="inlineStr">
-        <is>
-          <t>Number of outstanding loans</t>
-        </is>
-      </c>
-      <c r="D237" s="2" t="inlineStr">
-        <is>
           <t>6.10. Combien de crédit en cours, non totalement remboursés [NOM] a-t-il?</t>
         </is>
       </c>
     </row>
+    <row r="237"/>
+    <row r="238">
+      <c r="A238" s="6" t="inlineStr">
+        <is>
+          <t>Section 13 Part 2 — Remittances Received  |  Dataset: s13_2_me_ben2021</t>
+        </is>
+      </c>
+    </row>
     <row r="239">
-      <c r="A239" s="6" t="inlineStr">
-        <is>
-          <t>Section 13 Part 2 — Remittances Received  |  Dataset: s13_2_me_sen2021</t>
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>Transfers/remittances received. Note: variable names differ from 2018 (s13q22a/b vs s13aq17a/b, s13q19 vs s13aq14).</t>
         </is>
       </c>
     </row>
     <row r="240">
-      <c r="A240" s="4" t="inlineStr">
-        <is>
-          <t>Transfers/remittances received. Note: variable names differ from 2018 (s13q22a/b vs s13aq17a/b, s13q19 vs s13aq14).</t>
+      <c r="A240" s="2" t="n"/>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>s13q19</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>Location of sender (was s13aq14 in 2018)</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>13.19. Quel est le lieu de résidence de l'expéditeur ?</t>
         </is>
       </c>
     </row>
@@ -8084,17 +8094,17 @@
       <c r="A241" s="2" t="n"/>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>s13q19</t>
+          <t>s13q22a</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Location of sender (was s13aq14 in 2018)</t>
+          <t>Amount sent each time (was s13aq17a in 2018)</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>13.19. Quel est le lieu de résidence de l'expéditeur ?</t>
+          <t>13.22a. Quelle est le montant envoyé à chaque fois?</t>
         </is>
       </c>
     </row>
@@ -8102,33 +8112,15 @@
       <c r="A242" s="2" t="n"/>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>s13q22a</t>
+          <t>s13q22b</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Amount sent each time (was s13aq17a in 2018)</t>
+          <t>Frequency of transfers (was s13aq17b in 2018)</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
-        <is>
-          <t>13.22a. Quelle est le montant envoyé à chaque fois?</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" s="2" t="n"/>
-      <c r="B243" s="2" t="inlineStr">
-        <is>
-          <t>s13q22b</t>
-        </is>
-      </c>
-      <c r="C243" s="2" t="inlineStr">
-        <is>
-          <t>Frequency of transfers (was s13aq17b in 2018)</t>
-        </is>
-      </c>
-      <c r="D243" s="2" t="inlineStr">
         <is>
           <t>13.22b. Quelle est la fréquence des transferts envoyés à chaque fois?</t>
         </is>
@@ -8137,24 +8129,24 @@
   </sheetData>
   <mergeCells count="22">
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A188:D188"/>
-    <mergeCell ref="A240:D240"/>
     <mergeCell ref="A156:D156"/>
-    <mergeCell ref="A230:D230"/>
     <mergeCell ref="A229:D229"/>
+    <mergeCell ref="A114:D114"/>
     <mergeCell ref="A77:D77"/>
-    <mergeCell ref="A114:D114"/>
     <mergeCell ref="A157:D157"/>
     <mergeCell ref="A98:D98"/>
+    <mergeCell ref="A191:D191"/>
     <mergeCell ref="A138:D138"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A228:D228"/>
     <mergeCell ref="A78:D78"/>
-    <mergeCell ref="A187:D187"/>
     <mergeCell ref="A65:D65"/>
     <mergeCell ref="A137:D137"/>
     <mergeCell ref="A99:D99"/>
     <mergeCell ref="A66:D66"/>
+    <mergeCell ref="A192:D192"/>
+    <mergeCell ref="A238:D238"/>
     <mergeCell ref="A239:D239"/>
     <mergeCell ref="A113:D113"/>
     <mergeCell ref="A2:D2"/>

</xml_diff>